<commit_message>
chore: save latest app updates
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/onepop_社會橫幅_全冊_學期版.xlsx
+++ b/onepop_社會橫幅_全冊_學期版.xlsx
@@ -2911,7 +2911,6 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
@@ -4480,7 +4479,6 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
@@ -10696,7 +10694,7 @@
       <c r="D5" s="17" t="inlineStr">
         <is>
           <t>日治統治三階段：
-① 無方針主義（1895-1919）：軍事鎮壓、差別法律
+① 漸進主義（1895-1919）：軍事鎮壓、差別法律
 ② 內地延長主義（1919-1937）：同化政策、推行日語
 ③ 皇民化運動（1937-1945）：改姓名、參拜神社
 口訣：鎮壓→同化→皇民</t>
@@ -21195,7 +21193,7 @@
           <t>1911辛亥革命 → 推翻清朝、結束帝制
 孫中山就任臨時大總統（南京）
 中華民國元年 = 1912年
-⚠️ 辛亥革命 = 亞洲第一個民主共和國的誕生</t>
+⚠️ 辛亥革命 = 中國歷史上第一個民主共和國的誕生</t>
         </is>
       </c>
       <c r="E3" t="n">

</xml_diff>